<commit_message>
Built site for gh-pages
</commit_message>
<xml_diff>
--- a/posts/data/生存時間例データ.xlsx
+++ b/posts/data/生存時間例データ.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wopi.dropbox.com/wopi/files/oid_12106801812261828096/WOPIServiceId_TP_DROPBOX_PLUS/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{BE47067C-A23F-4B18-9985-2104B1B6B53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95B7E74E-6BB9-4985-AFD3-14C9D20B571E}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{BE47067C-A23F-4B18-9985-2104B1B6B53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{877DB034-DA1F-44FB-81E5-940D19EAF660}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{D509D36E-044D-44D3-B470-BDC212007F12}"/>
   </bookViews>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A7">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -1089,7 +1089,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A9">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -1100,7 +1100,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.7">
       <c r="A10">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B10">
         <v>1</v>

</xml_diff>